<commit_message>
Accept a government ID on file for TFS-sourced deals, add the upload templates of the new masters, and align the suites with duplicate control
</commit_message>
<xml_diff>
--- a/docs/package/05_Delivery/Upload_Templates/Account_Category_Upload_Template.xlsx
+++ b/docs/package/05_Delivery/Upload_Templates/Account_Category_Upload_Template.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="46">
   <si>
     <t xml:space="preserve">Account Category Code</t>
   </si>
@@ -99,12 +99,6 @@
     <t xml:space="preserve">Master &gt; Finance &gt; Account Category (no Upload button on this screen yet: a System Administrator uploads the file through the API route)</t>
   </si>
   <si>
-    <t xml:space="preserve">API route</t>
-  </si>
-  <si>
-    <t xml:space="preserve">POST /api/masters/account-category/upload (multipart field "file")</t>
-  </si>
-  <si>
     <t xml:space="preserve">File types</t>
   </si>
   <si>
@@ -135,10 +129,10 @@
     <t xml:space="preserve">The rows under the header on the Data sheet are samples. Delete them before you upload your own data.</t>
   </si>
   <si>
-    <t xml:space="preserve">Dates and amounts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enter dates as YYYY-MM-DD and amounts as plain numbers (no peso sign, no thousands separator). The Data sheet cells are formatted as text so that Excel keeps what you type.</t>
+    <t xml:space="preserve">Amounts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter amounts as plain numbers (no peso sign, no thousands separator). The Data sheet cells are formatted as text so that Excel keeps what you type.</t>
   </si>
   <si>
     <t xml:space="preserve">What happens on errors</t>
@@ -153,10 +147,10 @@
     <t xml:space="preserve">Each row creates a new record, checked exactly like Add on the screen. A row whose code already exists is refused (edit existing records on the screen).</t>
   </si>
   <si>
-    <t xml:space="preserve">Source</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generated by backend/scripts/build-upload-templates.js from the column list the importer itself uses. Do not rename the headers.</t>
+    <t xml:space="preserve">Headers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The headers are the ones the import reads. Do not rename them.</t>
   </si>
 </sst>
 </file>
@@ -164,9 +158,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -193,8 +187,42 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF0B2A4A"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF5F6B76"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -222,6 +250,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF4CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -253,9 +299,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -276,6 +322,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -432,7 +485,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -535,14 +588,6 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>